<commit_message>
Attention window January 2020 - December 2025 for page views and news mentions (news on the union of 244 Media Cloud national collections); inputs and expected outputs refreshed from the paper; criteria table label updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UX2ofEzNyc9hLtSVWNL9f
</commit_message>
<xml_diff>
--- a/data/mainPrizeList_pre-imputation.xlsx
+++ b/data/mainPrizeList_pre-imputation.xlsx
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>661.167463218669</v>
+        <v>659.9248144414286</v>
       </c>
       <c r="C2" t="n">
         <v>0.82</v>
@@ -683,13 +683,13 @@
         <v>4</v>
       </c>
       <c r="AC2" t="n">
-        <v>6.495518489533723</v>
+        <v>6.493640088210396</v>
       </c>
       <c r="AD2" t="n">
-        <v>3608</v>
+        <v>1911</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.191186004642789</v>
+        <v>7.555905093611346</v>
       </c>
     </row>
     <row r="3">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>479.005694261936</v>
+        <v>466.5713060300773</v>
       </c>
       <c r="C3" t="n">
         <v>0.97</v>
@@ -790,13 +790,13 @@
         <v>8</v>
       </c>
       <c r="AC3" t="n">
-        <v>6.173797966877271</v>
+        <v>6.147551863365338</v>
       </c>
       <c r="AD3" t="n">
-        <v>492</v>
+        <v>288</v>
       </c>
       <c r="AE3" t="n">
-        <v>6.20050917404269</v>
+        <v>5.666426688112432</v>
       </c>
     </row>
     <row r="4">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37.3631187034604</v>
+        <v>35.40343480800117</v>
       </c>
       <c r="C4" t="n">
         <v>0.51</v>
@@ -897,13 +897,13 @@
         <v>9</v>
       </c>
       <c r="AC4" t="n">
-        <v>3.647096547634907</v>
+        <v>3.594663133047976</v>
       </c>
       <c r="AD4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AE4" t="n">
-        <v>3.091042453358316</v>
+        <v>3.178053830347946</v>
       </c>
     </row>
     <row r="5">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54.49926345404897</v>
+        <v>53.68224881540364</v>
       </c>
       <c r="C5" t="n">
         <v>0.72</v>
@@ -1004,13 +1004,13 @@
         <v>7</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.016369749566111</v>
+        <v>4.001539137846268</v>
       </c>
       <c r="AD5" t="n">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="AE5" t="n">
-        <v>4.0943445622221</v>
+        <v>3.258096538021482</v>
       </c>
     </row>
     <row r="6">
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.882437697397238</v>
+        <v>0.9323798459946548</v>
       </c>
       <c r="C6" t="n">
         <v>0.57</v>
@@ -1111,13 +1111,13 @@
         <v>5</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.6325675844721199</v>
+        <v>0.6587523241232625</v>
       </c>
       <c r="AD6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>1.09861228866811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>4.07643907869762</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
@@ -1216,13 +1216,13 @@
         <v>9</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.6094379124341</v>
+        <v>1.624610047036609</v>
       </c>
       <c r="AD7" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="AE7" t="n">
-        <v>2.772588722239781</v>
+        <v>1.945910149055313</v>
       </c>
     </row>
     <row r="8">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>4.07643907869762</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
@@ -1321,13 +1321,13 @@
         <v>7</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.6094379124341</v>
+        <v>1.624610047036609</v>
       </c>
       <c r="AD8" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="AE8" t="n">
-        <v>3.713572066704308</v>
+        <v>3.091042453358316</v>
       </c>
     </row>
     <row r="9">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>4.07643907869762</v>
       </c>
       <c r="C9" t="n">
         <v>0.59</v>
@@ -1428,13 +1428,13 @@
         <v>5</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.6094379124341</v>
+        <v>1.624610047036609</v>
       </c>
       <c r="AD9" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="AE9" t="n">
-        <v>2.995732273553991</v>
+        <v>2.772588722239781</v>
       </c>
     </row>
     <row r="10">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>4.07643907869762</v>
       </c>
       <c r="C10" t="n">
         <v>0.61</v>
@@ -1535,13 +1535,13 @@
         <v>6</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.6094379124341</v>
+        <v>1.624610047036609</v>
       </c>
       <c r="AD10" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="AE10" t="n">
-        <v>2.639057329615258</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="11">
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>4.07643907869762</v>
       </c>
       <c r="C11" t="n">
         <v>0.44</v>
@@ -1642,13 +1642,13 @@
         <v>11</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.6094379124341</v>
+        <v>1.624610047036609</v>
       </c>
       <c r="AD11" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AE11" t="n">
-        <v>3.433987204485146</v>
+        <v>3.49650756146648</v>
       </c>
     </row>
     <row r="12">
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26.0783450294033</v>
+        <v>26.46712776330084</v>
       </c>
       <c r="C12" t="n">
         <v>0.47</v>
@@ -1749,13 +1749,13 @@
         <v>9</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.298734332048144</v>
+        <v>3.312989935605225</v>
       </c>
       <c r="AD12" t="n">
-        <v>347</v>
+        <v>114</v>
       </c>
       <c r="AE12" t="n">
-        <v>5.852202479774474</v>
+        <v>4.74493212836325</v>
       </c>
     </row>
     <row r="13">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C13" t="n">
         <v>0.47</v>
@@ -1856,13 +1856,13 @@
         <v>3</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD13" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="AE13" t="n">
-        <v>4.060443010546419</v>
+        <v>2.890371757896165</v>
       </c>
     </row>
     <row r="14">
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C14" t="n">
         <v>0.58</v>
@@ -1963,13 +1963,13 @@
         <v>4</v>
       </c>
       <c r="AC14" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD14" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AE14" t="n">
-        <v>2.70805020110221</v>
+        <v>1.945910149055313</v>
       </c>
     </row>
     <row r="15">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C15" t="n">
         <v>0.39</v>
@@ -2070,13 +2070,13 @@
         <v>7</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD15" t="n">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="AE15" t="n">
-        <v>4.406719247264253</v>
+        <v>3.555348061489414</v>
       </c>
     </row>
     <row r="16">
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
@@ -2175,13 +2175,13 @@
         <v>4</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD16" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="AE16" t="n">
-        <v>3.713572066704308</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="17">
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C17" t="n">
         <v>0.5</v>
@@ -2282,13 +2282,13 @@
         <v>4</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD17" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AE17" t="n">
-        <v>2.19722457733622</v>
+        <v>0.6931471805599453</v>
       </c>
     </row>
     <row r="18">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>14.9200613228209</v>
+        <v>13.90704847422981</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
@@ -2387,13 +2387,13 @@
         <v>6</v>
       </c>
       <c r="AC18" t="n">
-        <v>2.767580032344804</v>
+        <v>2.70183415305934</v>
       </c>
       <c r="AD18" t="n">
-        <v>152</v>
+        <v>1093</v>
       </c>
       <c r="AE18" t="n">
-        <v>5.030437921392435</v>
+        <v>6.997595982981927</v>
       </c>
     </row>
     <row r="19">
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4.601490578823033</v>
+        <v>4.560384170032933</v>
       </c>
       <c r="C19" t="n">
         <v>0.37</v>
@@ -2494,13 +2494,13 @@
         <v>9</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.723032737112706</v>
+        <v>1.715667201205183</v>
       </c>
       <c r="AD19" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="AE19" t="n">
-        <v>3.295836866004329</v>
+        <v>2.079441541679836</v>
       </c>
     </row>
     <row r="20">
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17.0730731874536</v>
+        <v>16.87485510267497</v>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="n">
@@ -2599,13 +2599,13 @@
         <v>7</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.894423161391786</v>
+        <v>2.883394982403159</v>
       </c>
       <c r="AD20" t="n">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="AE20" t="n">
-        <v>4.248495242049359</v>
+        <v>3.871201010907891</v>
       </c>
     </row>
     <row r="21">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>96.1593413560182</v>
+        <v>99.0730557301288</v>
       </c>
       <c r="C21" t="n">
         <v>0.55</v>
@@ -2706,13 +2706,13 @@
         <v>10</v>
       </c>
       <c r="AC21" t="n">
-        <v>4.576352325148646</v>
+        <v>4.605900476562293</v>
       </c>
       <c r="AD21" t="n">
-        <v>208</v>
+        <v>173</v>
       </c>
       <c r="AE21" t="n">
-        <v>5.342334251964811</v>
+        <v>5.159055299214529</v>
       </c>
     </row>
     <row r="22">
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>58.0203345286087</v>
+        <v>60.15539047542666</v>
       </c>
       <c r="C22" t="n">
         <v>0.39</v>
@@ -2813,13 +2813,13 @@
         <v>7</v>
       </c>
       <c r="AC22" t="n">
-        <v>4.077882037553774</v>
+        <v>4.113418009931233</v>
       </c>
       <c r="AD22" t="n">
-        <v>344</v>
+        <v>217</v>
       </c>
       <c r="AE22" t="n">
-        <v>5.84354441703136</v>
+        <v>5.384495062789089</v>
       </c>
     </row>
     <row r="23">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>84.401826819698</v>
+        <v>90.16724187456281</v>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
@@ -2918,13 +2918,13 @@
         <v>8</v>
       </c>
       <c r="AC23" t="n">
-        <v>4.447367491897091</v>
+        <v>4.512695642584217</v>
       </c>
       <c r="AD23" t="n">
-        <v>151</v>
+        <v>62</v>
       </c>
       <c r="AE23" t="n">
-        <v>5.023880520846276</v>
+        <v>4.143134726391533</v>
       </c>
     </row>
     <row r="24">
@@ -2934,7 +2934,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>7.37078405606658</v>
+        <v>8.013031099430574</v>
       </c>
       <c r="C24" t="n">
         <v>0.58</v>
@@ -3025,13 +3025,13 @@
         <v>2</v>
       </c>
       <c r="AC24" t="n">
-        <v>2.124747554674122</v>
+        <v>2.198671430076538</v>
       </c>
       <c r="AD24" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AE24" t="n">
-        <v>2.19722457733622</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="25">
@@ -3135,10 +3135,10 @@
         <v>2.079441541679836</v>
       </c>
       <c r="AD25" t="n">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="AE25" t="n">
-        <v>5.135798437050262</v>
+        <v>4.02535169073515</v>
       </c>
     </row>
     <row r="26">
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>26.5254051686378</v>
+        <v>26.29462330267192</v>
       </c>
       <c r="C26" t="n">
         <v>0.6</v>
@@ -3239,13 +3239,13 @@
         <v>7</v>
       </c>
       <c r="AC26" t="n">
-        <v>3.315109402523577</v>
+        <v>3.306689734173911</v>
       </c>
       <c r="AD26" t="n">
-        <v>257</v>
+        <v>96</v>
       </c>
       <c r="AE26" t="n">
-        <v>5.552959584921617</v>
+        <v>4.574710978503383</v>
       </c>
     </row>
     <row r="27">
@@ -3255,7 +3255,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>26.1286823981137</v>
+        <v>25.89872237936504</v>
       </c>
       <c r="C27" t="n">
         <v>0.5600000000000001</v>
@@ -3346,13 +3346,13 @@
         <v>4</v>
       </c>
       <c r="AC27" t="n">
-        <v>3.300591559259015</v>
+        <v>3.29207879028897</v>
       </c>
       <c r="AD27" t="n">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="AE27" t="n">
-        <v>4.369447852467021</v>
+        <v>3.610917912644224</v>
       </c>
     </row>
     <row r="28">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>127.703206084768</v>
+        <v>125.0872850490431</v>
       </c>
       <c r="C28" t="n">
         <v>0.46</v>
@@ -3453,13 +3453,13 @@
         <v>9</v>
       </c>
       <c r="AC28" t="n">
-        <v>4.857509025595358</v>
+        <v>4.836974405603398</v>
       </c>
       <c r="AD28" t="n">
-        <v>142</v>
+        <v>43</v>
       </c>
       <c r="AE28" t="n">
-        <v>4.962844630259907</v>
+        <v>3.784189633918261</v>
       </c>
     </row>
     <row r="29">
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9.11300919842312</v>
+        <v>9.671302379909475</v>
       </c>
       <c r="C29" t="n">
         <v>0.77</v>
@@ -3560,13 +3560,13 @@
         <v>2</v>
       </c>
       <c r="AC29" t="n">
-        <v>2.313822634483856</v>
+        <v>2.367558117837722</v>
       </c>
       <c r="AD29" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="AE29" t="n">
-        <v>2.639057329615258</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="30">
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9.11300919842312</v>
+        <v>9.671302379909475</v>
       </c>
       <c r="C30" t="n">
         <v>0.52</v>
@@ -3667,13 +3667,13 @@
         <v>7</v>
       </c>
       <c r="AC30" t="n">
-        <v>2.313822634483856</v>
+        <v>2.367558117837722</v>
       </c>
       <c r="AD30" t="n">
-        <v>155</v>
+        <v>31</v>
       </c>
       <c r="AE30" t="n">
-        <v>5.049856007249537</v>
+        <v>3.465735902799727</v>
       </c>
     </row>
     <row r="31">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>9.11300919842312</v>
+        <v>9.671302379909475</v>
       </c>
       <c r="C31" t="n">
         <v>0.85</v>
@@ -3774,13 +3774,13 @@
         <v>5</v>
       </c>
       <c r="AC31" t="n">
-        <v>2.313822634483856</v>
+        <v>2.367558117837722</v>
       </c>
       <c r="AD31" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE31" t="n">
-        <v>2.302585092994046</v>
+        <v>0.6931471805599453</v>
       </c>
     </row>
     <row r="32">
@@ -3790,7 +3790,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>9.11300919842312</v>
+        <v>9.671302379909475</v>
       </c>
       <c r="C32" t="n">
         <v>0.78</v>
@@ -3881,13 +3881,13 @@
         <v>8</v>
       </c>
       <c r="AC32" t="n">
-        <v>2.313822634483856</v>
+        <v>2.367558117837722</v>
       </c>
       <c r="AD32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE32" t="n">
-        <v>1.386294361119891</v>
+        <v>0.6931471805599453</v>
       </c>
     </row>
     <row r="33">
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>9.11300919842312</v>
+        <v>9.671302379909475</v>
       </c>
       <c r="C33" t="n">
         <v>0.3</v>
@@ -3988,13 +3988,13 @@
         <v>7</v>
       </c>
       <c r="AC33" t="n">
-        <v>2.313822634483856</v>
+        <v>2.367558117837722</v>
       </c>
       <c r="AD33" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AE33" t="n">
-        <v>2.302585092994046</v>
+        <v>1.945910149055313</v>
       </c>
     </row>
     <row r="34">
@@ -4004,7 +4004,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>16</v>
+        <v>15.03504161191415</v>
       </c>
       <c r="C34" t="n">
         <v>0.55</v>
@@ -4095,13 +4095,13 @@
         <v>6</v>
       </c>
       <c r="AC34" t="n">
-        <v>2.833213344056216</v>
+        <v>2.774776428209675</v>
       </c>
       <c r="AD34" t="n">
-        <v>266</v>
+        <v>317</v>
       </c>
       <c r="AE34" t="n">
-        <v>5.58724865840025</v>
+        <v>5.762051382780177</v>
       </c>
     </row>
     <row r="35">
@@ -4111,7 +4111,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6.07393154370815</v>
+        <v>6.164113696288853</v>
       </c>
       <c r="C35" t="n">
         <v>0.52</v>
@@ -4202,13 +4202,13 @@
         <v>11</v>
       </c>
       <c r="AC35" t="n">
-        <v>1.956416413567699</v>
+        <v>1.969084354576279</v>
       </c>
       <c r="AD35" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="AE35" t="n">
-        <v>3.258096538021482</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="36">
@@ -4218,7 +4218,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8.592860271572491</v>
+        <v>9.521462987297417</v>
       </c>
       <c r="C36" t="n">
         <v>0.51</v>
@@ -4309,13 +4309,13 @@
         <v>3</v>
       </c>
       <c r="AC36" t="n">
-        <v>2.2610191000644</v>
+        <v>2.353417264874207</v>
       </c>
       <c r="AD36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AE36" t="n">
-        <v>1.386294361119891</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1107.29852139757</v>
+        <v>1109.038732118723</v>
       </c>
       <c r="C37" t="n">
         <v>0.95</v>
@@ -4416,13 +4416,13 @@
         <v>8</v>
       </c>
       <c r="AC37" t="n">
-        <v>7.010581254663213</v>
+        <v>7.012150187498257</v>
       </c>
       <c r="AD37" t="n">
-        <v>1370</v>
+        <v>779</v>
       </c>
       <c r="AE37" t="n">
-        <v>7.223295679562314</v>
+        <v>6.659293919683638</v>
       </c>
     </row>
     <row r="38">
@@ -4432,7 +4432,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>28.1474310584244</v>
+        <v>27.6333129427402</v>
       </c>
       <c r="C38" t="n">
         <v>0.64</v>
@@ -4523,13 +4523,13 @@
         <v>2</v>
       </c>
       <c r="AC38" t="n">
-        <v>3.372366780557031</v>
+        <v>3.354570828194031</v>
       </c>
       <c r="AD38" t="n">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="AE38" t="n">
-        <v>4.442651256490317</v>
+        <v>3.526360524616162</v>
       </c>
     </row>
     <row r="39">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>9.53679369250986</v>
+        <v>9.789294057526646</v>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
@@ -4628,13 +4628,13 @@
         <v>2</v>
       </c>
       <c r="AC39" t="n">
-        <v>2.354873293087178</v>
+        <v>2.378554351506584</v>
       </c>
       <c r="AD39" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="AE39" t="n">
-        <v>3.13549421592915</v>
+        <v>2.639057329615258</v>
       </c>
     </row>
     <row r="40">
@@ -4644,7 +4644,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4.19294787560228</v>
+        <v>4.149784640093444</v>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="n">
@@ -4733,13 +4733,13 @@
         <v>7</v>
       </c>
       <c r="AC40" t="n">
-        <v>1.647301527377237</v>
+        <v>1.638954896343687</v>
       </c>
       <c r="AD40" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="AE40" t="n">
-        <v>2.995732273553991</v>
+        <v>1.6094379124341</v>
       </c>
     </row>
     <row r="41">
@@ -4749,7 +4749,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6.13198000211458</v>
+        <v>6.263570802828358</v>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
@@ -4838,13 +4838,13 @@
         <v>7</v>
       </c>
       <c r="AC41" t="n">
-        <v>1.964588896030976</v>
+        <v>1.982871554039657</v>
       </c>
       <c r="AD41" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE41" t="n">
-        <v>2.639057329615258</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -4854,7 +4854,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>80.3143965745419</v>
+        <v>82.59750185301101</v>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
@@ -4943,13 +4943,13 @@
         <v>4</v>
       </c>
       <c r="AC42" t="n">
-        <v>4.398323080514678</v>
+        <v>4.426013637503159</v>
       </c>
       <c r="AD42" t="n">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="AE42" t="n">
-        <v>4.290459441148391</v>
+        <v>3.688879454113936</v>
       </c>
     </row>
     <row r="43">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>15.8086946999562</v>
+        <v>15.62910643889619</v>
       </c>
       <c r="C43" t="n">
         <v>0.4</v>
@@ -5050,13 +5050,13 @@
         <v>9</v>
       </c>
       <c r="AC43" t="n">
-        <v>2.821896294194775</v>
+        <v>2.811154559884871</v>
       </c>
       <c r="AD43" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="AE43" t="n">
-        <v>2.484906649788</v>
+        <v>1.945910149055313</v>
       </c>
     </row>
     <row r="44">
@@ -5066,7 +5066,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.090909090909091</v>
+        <v>1.111250344658096</v>
       </c>
       <c r="C44" t="n">
         <v>0.41</v>
@@ -5157,13 +5157,13 @@
         <v>7</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.7375989431307791</v>
+        <v>0.7472803523882174</v>
       </c>
       <c r="AD44" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="AE44" t="n">
-        <v>2.833213344056216</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="45">
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1.090909090909091</v>
+        <v>1.111250344658096</v>
       </c>
       <c r="C45" t="n">
         <v>0.55</v>
@@ -5264,13 +5264,13 @@
         <v>6</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.7375989431307791</v>
+        <v>0.7472803523882174</v>
       </c>
       <c r="AD45" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="AE45" t="n">
-        <v>2.564949357461537</v>
+        <v>1.386294361119891</v>
       </c>
     </row>
     <row r="46">
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.090909090909091</v>
+        <v>1.111250344658096</v>
       </c>
       <c r="C46" t="n">
         <v>0.44</v>
@@ -5371,13 +5371,13 @@
         <v>7</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.7375989431307791</v>
+        <v>0.7472803523882174</v>
       </c>
       <c r="AD46" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="AE46" t="n">
-        <v>3.044522437723423</v>
+        <v>1.386294361119891</v>
       </c>
     </row>
     <row r="47">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>59.8817843348067</v>
+        <v>53.37060415493398</v>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="n">
@@ -5476,13 +5476,13 @@
         <v>8</v>
       </c>
       <c r="AC47" t="n">
-        <v>4.108934022171345</v>
+        <v>3.995823643013215</v>
       </c>
       <c r="AD47" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="AE47" t="n">
-        <v>4.110873864173311</v>
+        <v>3.761200115693562</v>
       </c>
     </row>
     <row r="48">
@@ -5492,7 +5492,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>42.1966710468681</v>
+        <v>43.18650532924514</v>
       </c>
       <c r="C48" t="n">
         <v>0.68</v>
@@ -5583,13 +5583,13 @@
         <v>4</v>
       </c>
       <c r="AC48" t="n">
-        <v>3.765763433180584</v>
+        <v>3.788419433174186</v>
       </c>
       <c r="AD48" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="AE48" t="n">
-        <v>3.761200115693562</v>
+        <v>3.091042453358316</v>
       </c>
     </row>
     <row r="49">
@@ -5599,7 +5599,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3.49206586230239</v>
+        <v>3.425083300100461</v>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
@@ -5688,13 +5688,13 @@
         <v>7</v>
       </c>
       <c r="AC49" t="n">
-        <v>1.502312698901921</v>
+        <v>1.487289103164167</v>
       </c>
       <c r="AD49" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="AE49" t="n">
-        <v>2.890371757896165</v>
+        <v>2.397895272798371</v>
       </c>
     </row>
     <row r="50">
@@ -5704,7 +5704,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.84357669435845</v>
+        <v>2.702772800001161</v>
       </c>
       <c r="C50" t="n">
         <v>0.5</v>
@@ -5795,13 +5795,13 @@
         <v>4</v>
       </c>
       <c r="AC50" t="n">
-        <v>1.34640336390963</v>
+        <v>1.309081944391879</v>
       </c>
       <c r="AD50" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="AE50" t="n">
-        <v>3.332204510175204</v>
+        <v>1.945910149055313</v>
       </c>
     </row>
     <row r="51">
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17.4384090035489</v>
+        <v>16.81094553710126</v>
       </c>
       <c r="C51" t="n">
         <v>0.57</v>
@@ -5902,13 +5902,13 @@
         <v>10</v>
       </c>
       <c r="AC51" t="n">
-        <v>2.914435934772138</v>
+        <v>2.879813186128227</v>
       </c>
       <c r="AD51" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="AE51" t="n">
-        <v>2.484906649788</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="52">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.92378449408673</v>
+        <v>3.015038691779821</v>
       </c>
       <c r="C52" t="n">
         <v>0.48</v>
@@ -6009,13 +6009,13 @@
         <v>2</v>
       </c>
       <c r="AC52" t="n">
-        <v>1.36705662023745</v>
+        <v>1.390046984159221</v>
       </c>
       <c r="AD52" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="AE52" t="n">
-        <v>2.484906649788</v>
+        <v>1.791759469228055</v>
       </c>
     </row>
     <row r="53">
@@ -6025,7 +6025,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>41.4361585632939</v>
+        <v>40.16097240473061</v>
       </c>
       <c r="C53" t="n">
         <v>0.66</v>
@@ -6116,13 +6116,13 @@
         <v>9</v>
       </c>
       <c r="AC53" t="n">
-        <v>3.748000795117849</v>
+        <v>3.717490535680238</v>
       </c>
       <c r="AD53" t="n">
-        <v>624</v>
+        <v>351</v>
       </c>
       <c r="AE53" t="n">
-        <v>6.437751649736401</v>
+        <v>5.863631175598097</v>
       </c>
     </row>
     <row r="54">
@@ -6132,7 +6132,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>14.00313914440063</v>
+        <v>13.93755779432521</v>
       </c>
       <c r="C54" t="n">
         <v>0.72</v>
@@ -6223,13 +6223,13 @@
         <v>2</v>
       </c>
       <c r="AC54" t="n">
-        <v>2.708259455500357</v>
+        <v>2.703878698760409</v>
       </c>
       <c r="AD54" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="AE54" t="n">
-        <v>2.70805020110221</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="55">
@@ -6239,7 +6239,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>14.00313914440063</v>
+        <v>13.93755779432521</v>
       </c>
       <c r="C55" t="n">
         <v>0.62</v>
@@ -6330,13 +6330,13 @@
         <v>4</v>
       </c>
       <c r="AC55" t="n">
-        <v>2.708259455500357</v>
+        <v>2.703878698760409</v>
       </c>
       <c r="AD55" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="AE55" t="n">
-        <v>3.761200115693562</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="56">
@@ -6346,7 +6346,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>14.00313914440063</v>
+        <v>13.93755779432521</v>
       </c>
       <c r="C56" t="n">
         <v>0.55</v>
@@ -6437,13 +6437,13 @@
         <v>7</v>
       </c>
       <c r="AC56" t="n">
-        <v>2.708259455500357</v>
+        <v>2.703878698760409</v>
       </c>
       <c r="AD56" t="n">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="AE56" t="n">
-        <v>4.189654742026425</v>
+        <v>3.13549421592915</v>
       </c>
     </row>
     <row r="57">
@@ -6453,7 +6453,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5.09691195795006</v>
+        <v>5.05457001022047</v>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="n">
@@ -6542,13 +6542,13 @@
         <v>7</v>
       </c>
       <c r="AC57" t="n">
-        <v>1.807782406596727</v>
+        <v>1.800813360481868</v>
       </c>
       <c r="AD57" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AE57" t="n">
-        <v>2.772588722239781</v>
+        <v>2.079441541679836</v>
       </c>
     </row>
     <row r="58">
@@ -6558,7 +6558,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>17.75699267880608</v>
+        <v>16.82588122737856</v>
       </c>
       <c r="C58" t="n">
         <v>0.5</v>
@@ -6649,13 +6649,13 @@
         <v>9</v>
       </c>
       <c r="AC58" t="n">
-        <v>2.931566625760171</v>
+        <v>2.880651402799453</v>
       </c>
       <c r="AD58" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="AE58" t="n">
-        <v>3.178053830347946</v>
+        <v>3.332204510175204</v>
       </c>
     </row>
     <row r="59">
@@ -6665,7 +6665,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>27.11520997217333</v>
+        <v>27.9497571478589</v>
       </c>
       <c r="C59" t="n">
         <v>0.63</v>
@@ -6756,13 +6756,13 @@
         <v>4</v>
       </c>
       <c r="AC59" t="n">
-        <v>3.336310710048958</v>
+        <v>3.365561815308824</v>
       </c>
       <c r="AD59" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AE59" t="n">
-        <v>2.079441541679836</v>
+        <v>1.791759469228055</v>
       </c>
     </row>
     <row r="60">
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>47.11520997217333</v>
+        <v>45.11330292096446</v>
       </c>
       <c r="C60" t="n">
         <v>0.66</v>
@@ -6863,13 +6863,13 @@
         <v>9</v>
       </c>
       <c r="AC60" t="n">
-        <v>3.873598342763787</v>
+        <v>3.831101474990546</v>
       </c>
       <c r="AD60" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AE60" t="n">
-        <v>2.639057329615258</v>
+        <v>2.484906649788</v>
       </c>
     </row>
     <row r="61">
@@ -6879,7 +6879,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>47.49926345404897</v>
+        <v>52.71865746408639</v>
       </c>
       <c r="C61" t="n">
         <v>0.6</v>
@@ -6970,13 +6970,13 @@
         <v>7</v>
       </c>
       <c r="AC61" t="n">
-        <v>3.881548611313667</v>
+        <v>3.983760379981735</v>
       </c>
       <c r="AD61" t="n">
-        <v>130</v>
+        <v>79</v>
       </c>
       <c r="AE61" t="n">
-        <v>4.875197323201151</v>
+        <v>4.382026634673881</v>
       </c>
     </row>
     <row r="62">
@@ -6986,7 +6986,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>13.4959483136224</v>
+        <v>13.51383413637027</v>
       </c>
       <c r="C62" t="n">
         <v>0.54</v>
@@ -7077,13 +7077,13 @@
         <v>10</v>
       </c>
       <c r="AC62" t="n">
-        <v>2.673869183732898</v>
+        <v>2.675102272953405</v>
       </c>
       <c r="AD62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AE62" t="n">
-        <v>1.945910149055313</v>
+        <v>0.6931471805599453</v>
       </c>
     </row>
     <row r="63">
@@ -7093,7 +7093,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>16.1486470044289</v>
+        <v>15.53992300953536</v>
       </c>
       <c r="C63" t="n">
         <v>0.43</v>
@@ -7184,13 +7184,13 @@
         <v>7</v>
       </c>
       <c r="AC63" t="n">
-        <v>2.841919278629787</v>
+        <v>2.80577703478032</v>
       </c>
       <c r="AD63" t="n">
-        <v>111</v>
+        <v>32</v>
       </c>
       <c r="AE63" t="n">
-        <v>4.718498871295094</v>
+        <v>3.49650756146648</v>
       </c>
     </row>
     <row r="64">
@@ -7200,7 +7200,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>43.7417871222076</v>
+        <v>41.53252299605781</v>
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="n">
@@ -7289,13 +7289,13 @@
         <v>4</v>
       </c>
       <c r="AC64" t="n">
-        <v>3.80090789988218</v>
+        <v>3.750269030244269</v>
       </c>
       <c r="AD64" t="n">
-        <v>119</v>
+        <v>55</v>
       </c>
       <c r="AE64" t="n">
-        <v>4.787491742782046</v>
+        <v>4.02535169073515</v>
       </c>
     </row>
     <row r="65">
@@ -7305,7 +7305,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>6.385352498288843</v>
+        <v>6.385352498288844</v>
       </c>
       <c r="C65" t="n">
         <v>0.53</v>
@@ -7399,10 +7399,10 @@
         <v>1.999498646501481</v>
       </c>
       <c r="AD65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE65" t="n">
-        <v>1.6094379124341</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="66">
@@ -7412,7 +7412,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>51.8949846692948</v>
+        <v>47.05933347934005</v>
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="n">
@@ -7501,13 +7501,13 @@
         <v>10</v>
       </c>
       <c r="AC66" t="n">
-        <v>3.96830852660591</v>
+        <v>3.872436361700711</v>
       </c>
       <c r="AD66" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE66" t="n">
-        <v>1.945910149055313</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>50.71123521682</v>
+        <v>49.28091692217842</v>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="n">
@@ -7606,13 +7606,13 @@
         <v>10</v>
       </c>
       <c r="AC67" t="n">
-        <v>3.94567507351057</v>
+        <v>3.917625619875942</v>
       </c>
       <c r="AD67" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="AE67" t="n">
-        <v>3.091042453358316</v>
+        <v>1.791759469228055</v>
       </c>
     </row>
     <row r="68">
@@ -7716,10 +7716,10 @@
         <v>0</v>
       </c>
       <c r="AD68" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AE68" t="n">
-        <v>2.19722457733622</v>
+        <v>0.6931471805599453</v>
       </c>
     </row>
     <row r="69">
@@ -7823,10 +7823,10 @@
         <v>0</v>
       </c>
       <c r="AD69" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AE69" t="n">
-        <v>1.791759469228055</v>
+        <v>2.302585092994046</v>
       </c>
     </row>
     <row r="70">
@@ -7836,7 +7836,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>39.2377098749726</v>
+        <v>38.8280821527034</v>
       </c>
       <c r="C70" t="n">
         <v>0.5</v>
@@ -7927,13 +7927,13 @@
         <v>4</v>
       </c>
       <c r="AC70" t="n">
-        <v>3.694804612516204</v>
+        <v>3.68457224521085</v>
       </c>
       <c r="AD70" t="n">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="AE70" t="n">
-        <v>5.236441962829949</v>
+        <v>4.927253685157205</v>
       </c>
     </row>
     <row r="71">
@@ -7943,7 +7943,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>567.938994558156</v>
+        <v>570.9641141317688</v>
       </c>
       <c r="C71" t="n">
         <v>1</v>
@@ -8034,13 +8034,13 @@
         <v>3</v>
       </c>
       <c r="AC71" t="n">
-        <v>6.343773213190596</v>
+        <v>6.349076251879844</v>
       </c>
       <c r="AD71" t="n">
-        <v>10196</v>
+        <v>4743</v>
       </c>
       <c r="AE71" t="n">
-        <v>9.229848838364227</v>
+        <v>8.464635940677562</v>
       </c>
     </row>
     <row r="72">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1137.11949287551</v>
+        <v>1137.876132923438</v>
       </c>
       <c r="C72" t="n">
         <v>1</v>
@@ -8141,13 +8141,13 @@
         <v>10</v>
       </c>
       <c r="AC72" t="n">
-        <v>7.037132611700707</v>
+        <v>7.037797206807702</v>
       </c>
       <c r="AD72" t="n">
-        <v>13787</v>
+        <v>6802</v>
       </c>
       <c r="AE72" t="n">
-        <v>9.531553927636756</v>
+        <v>8.825118970345061</v>
       </c>
     </row>
     <row r="73">
@@ -8157,7 +8157,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>730.5567071702729</v>
+        <v>730.3548559003171</v>
       </c>
       <c r="C73" t="n">
         <v>1</v>
@@ -8248,13 +8248,13 @@
         <v>7</v>
       </c>
       <c r="AC73" t="n">
-        <v>6.595174739219395</v>
+        <v>6.594898780950512</v>
       </c>
       <c r="AD73" t="n">
-        <v>10425</v>
+        <v>4733</v>
       </c>
       <c r="AE73" t="n">
-        <v>9.252057965328051</v>
+        <v>8.462525790073929</v>
       </c>
     </row>
     <row r="74">
@@ -8264,7 +8264,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>8.688879466780589</v>
+        <v>8.965516342323175</v>
       </c>
       <c r="C74" t="n">
         <v>0.44</v>
@@ -8355,13 +8355,13 @@
         <v>7</v>
       </c>
       <c r="AC74" t="n">
-        <v>2.270978781112936</v>
+        <v>2.299130767909249</v>
       </c>
       <c r="AD74" t="n">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="AE74" t="n">
-        <v>3.761200115693562</v>
+        <v>2.94443897916644</v>
       </c>
     </row>
     <row r="75">
@@ -8371,7 +8371,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>27.3732064402235</v>
+        <v>32.89615899900566</v>
       </c>
       <c r="C75" t="n">
         <v>0.51</v>
@@ -8462,13 +8462,13 @@
         <v>4</v>
       </c>
       <c r="AC75" t="n">
-        <v>3.345445264648665</v>
+        <v>3.523301704102897</v>
       </c>
       <c r="AD75" t="n">
-        <v>194</v>
+        <v>153</v>
       </c>
       <c r="AE75" t="n">
-        <v>5.272999558563747</v>
+        <v>5.03695260241363</v>
       </c>
     </row>
     <row r="76">
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>22.9809785280735</v>
+        <v>20.75969418773591</v>
       </c>
       <c r="C76" t="n">
         <v>0.49</v>
@@ -8569,13 +8569,13 @@
         <v>7</v>
       </c>
       <c r="AC76" t="n">
-        <v>3.177260954774895</v>
+        <v>3.080059368016555</v>
       </c>
       <c r="AD76" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="AE76" t="n">
-        <v>3.637586159726386</v>
+        <v>2.833213344056216</v>
       </c>
     </row>
     <row r="77">
@@ -8585,7 +8585,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>9.4578963610795</v>
+        <v>9.295868664874224</v>
       </c>
       <c r="C77" t="n">
         <v>0.52</v>
@@ -8676,13 +8676,13 @@
         <v>8</v>
       </c>
       <c r="AC77" t="n">
-        <v>2.347357325703399</v>
+        <v>2.331742714275621</v>
       </c>
       <c r="AD77" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AE77" t="n">
-        <v>2.19722457733622</v>
+        <v>1.6094379124341</v>
       </c>
     </row>
     <row r="78">
@@ -8692,7 +8692,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>5.97240473061761</v>
+        <v>5.925135056212585</v>
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
@@ -8781,13 +8781,13 @@
         <v>4</v>
       </c>
       <c r="AC78" t="n">
-        <v>1.941960176835999</v>
+        <v>1.935157554585405</v>
       </c>
       <c r="AD78" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AE78" t="n">
-        <v>1.791759469228055</v>
+        <v>1.09861228866811</v>
       </c>
     </row>
     <row r="79">
@@ -8797,7 +8797,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>22.33172725945393</v>
+        <v>22.68564145617365</v>
       </c>
       <c r="C79" t="n">
         <v>0.7</v>
@@ -8888,13 +8888,13 @@
         <v>2</v>
       </c>
       <c r="AC79" t="n">
-        <v>3.149814119274548</v>
+        <v>3.164869018811332</v>
       </c>
       <c r="AD79" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="AE79" t="n">
-        <v>3.526360524616162</v>
+        <v>3.332204510175204</v>
       </c>
     </row>
     <row r="80">
@@ -8904,7 +8904,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>22.33172725945393</v>
+        <v>22.68564145617365</v>
       </c>
       <c r="C80" t="n">
         <v>0.6</v>
@@ -8995,13 +8995,13 @@
         <v>7</v>
       </c>
       <c r="AC80" t="n">
-        <v>3.149814119274548</v>
+        <v>3.164869018811332</v>
       </c>
       <c r="AD80" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="AE80" t="n">
-        <v>3.737669618283368</v>
+        <v>3.332204510175204</v>
       </c>
     </row>
     <row r="81">
@@ -9011,7 +9011,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>22.33172725945393</v>
+        <v>22.68564145617365</v>
       </c>
       <c r="C81" t="n">
         <v>0.77</v>
@@ -9102,13 +9102,13 @@
         <v>8</v>
       </c>
       <c r="AC81" t="n">
-        <v>3.149814119274548</v>
+        <v>3.164869018811332</v>
       </c>
       <c r="AD81" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AE81" t="n">
-        <v>3.258096538021482</v>
+        <v>3.295836866004329</v>
       </c>
     </row>
     <row r="82">
@@ -9118,7 +9118,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>6.09546906804772</v>
+        <v>6.224383643076152</v>
       </c>
       <c r="C82" t="n">
         <v>0.5</v>
@@ -9209,13 +9209,13 @@
         <v>11</v>
       </c>
       <c r="AC82" t="n">
-        <v>1.959456420906971</v>
+        <v>1.977461921442688</v>
       </c>
       <c r="AD82" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE82" t="n">
-        <v>1.09861228866811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -9225,7 +9225,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>5.60868136890819</v>
+        <v>5.730511879408522</v>
       </c>
       <c r="C83" t="n">
         <v>0.51</v>
@@ -9316,13 +9316,13 @@
         <v>11</v>
       </c>
       <c r="AC83" t="n">
-        <v>1.888384143631162</v>
+        <v>1.906651200111748</v>
       </c>
       <c r="AD83" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="AE83" t="n">
-        <v>3.663561646129646</v>
+        <v>2.890371757896165</v>
       </c>
     </row>
     <row r="84">
@@ -9332,7 +9332,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>14.0095269382392</v>
+        <v>14.09466710468681</v>
       </c>
       <c r="C84" t="n">
         <v>0.6899999999999999</v>
@@ -9423,13 +9423,13 @@
         <v>6</v>
       </c>
       <c r="AC84" t="n">
-        <v>2.708685128708957</v>
+        <v>2.714341509565958</v>
       </c>
       <c r="AD84" t="n">
-        <v>261</v>
+        <v>208</v>
       </c>
       <c r="AE84" t="n">
-        <v>5.568344503761097</v>
+        <v>5.342334251964811</v>
       </c>
     </row>
     <row r="85">
@@ -9439,7 +9439,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>853.04487725255</v>
+        <v>844.3599512634579</v>
       </c>
       <c r="C85" t="n">
         <v>1</v>
@@ -9530,13 +9530,13 @@
         <v>11</v>
       </c>
       <c r="AC85" t="n">
-        <v>6.749983741883948</v>
+        <v>6.739762514480955</v>
       </c>
       <c r="AD85" t="n">
-        <v>8221</v>
+        <v>3736</v>
       </c>
       <c r="AE85" t="n">
-        <v>9.014568767457824</v>
+        <v>8.226038429485484</v>
       </c>
     </row>
     <row r="86">
@@ -9546,7 +9546,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>9.261799167761724</v>
+        <v>9.039412687983647</v>
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="n">
@@ -9635,13 +9635,13 @@
         <v>7</v>
       </c>
       <c r="AC86" t="n">
-        <v>2.328428181850947</v>
+        <v>2.30651861533977</v>
       </c>
       <c r="AD86" t="n">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="AE86" t="n">
-        <v>4.912654885736052</v>
+        <v>4.653960350157523</v>
       </c>
     </row>
     <row r="87">
@@ -9651,7 +9651,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>128</v>
+        <v>120.3514434929557</v>
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="n">
@@ -9740,13 +9740,13 @@
         <v>9</v>
       </c>
       <c r="AC87" t="n">
-        <v>4.859812404361672</v>
+        <v>4.798690827387858</v>
       </c>
       <c r="AD87" t="n">
-        <v>1110</v>
+        <v>424</v>
       </c>
       <c r="AE87" t="n">
-        <v>7.01301578963963</v>
+        <v>6.052089168924417</v>
       </c>
     </row>
     <row r="88">
@@ -9756,7 +9756,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>13.8540297853701</v>
+        <v>13.90440210249671</v>
       </c>
       <c r="C88" t="n">
         <v>0.59</v>
@@ -9847,13 +9847,13 @@
         <v>4</v>
       </c>
       <c r="AC88" t="n">
-        <v>2.698271194453799</v>
+        <v>2.701656612437274</v>
       </c>
       <c r="AD88" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="AE88" t="n">
-        <v>3.555348061489414</v>
+        <v>1.791759469228055</v>
       </c>
     </row>
     <row r="89">
@@ -9863,7 +9863,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>33.3376114538557</v>
+        <v>30.90519473963837</v>
       </c>
       <c r="C89" t="n">
         <v>0.75</v>
@@ -9954,13 +9954,13 @@
         <v>6</v>
       </c>
       <c r="AC89" t="n">
-        <v>3.536241297251019</v>
+        <v>3.462768841035842</v>
       </c>
       <c r="AD89" t="n">
-        <v>509</v>
+        <v>462</v>
       </c>
       <c r="AE89" t="n">
-        <v>6.234410725718371</v>
+        <v>6.137727054086234</v>
       </c>
     </row>
     <row r="90">
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>11.6146517739816</v>
+        <v>11.85802671922908</v>
       </c>
       <c r="C90" t="n">
         <v>0.62</v>
@@ -10061,13 +10061,13 @@
         <v>5</v>
       </c>
       <c r="AC90" t="n">
-        <v>2.534858977588485</v>
+        <v>2.553968263741063</v>
       </c>
       <c r="AD90" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="AE90" t="n">
-        <v>3.178053830347946</v>
+        <v>2.19722457733622</v>
       </c>
     </row>
     <row r="91">
@@ -10077,7 +10077,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>4.41086289969339</v>
+        <v>4.367882172579939</v>
       </c>
       <c r="C91" t="n">
         <v>0.72</v>
@@ -10168,13 +10168,13 @@
         <v>6</v>
       </c>
       <c r="AC91" t="n">
-        <v>1.688408581007019</v>
+        <v>1.680433449461997</v>
       </c>
       <c r="AD91" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="AE91" t="n">
-        <v>3.737669618283368</v>
+        <v>3.178053830347946</v>
       </c>
     </row>
     <row r="92">
@@ -10184,7 +10184,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3</v>
+        <v>7.933639947437582</v>
       </c>
       <c r="C92" t="n">
         <v>0.68</v>
@@ -10275,13 +10275,13 @@
         <v>4</v>
       </c>
       <c r="AC92" t="n">
-        <v>1.386294361119891</v>
+        <v>2.189823920734055</v>
       </c>
       <c r="AD92" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AE92" t="n">
-        <v>2.564949357461537</v>
+        <v>1.6094379124341</v>
       </c>
     </row>
     <row r="93">
@@ -10291,7 +10291,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>7.49616732369689</v>
+        <v>7.444517447802599</v>
       </c>
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="n">
@@ -10380,13 +10380,13 @@
         <v>7</v>
       </c>
       <c r="AC93" t="n">
-        <v>2.139615158714419</v>
+        <v>2.133517408047261</v>
       </c>
       <c r="AD93" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="AE93" t="n">
-        <v>3.931825632724326</v>
+        <v>2.772588722239781</v>
       </c>
     </row>
     <row r="94">
@@ -10396,7 +10396,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>27.47276565028113</v>
+        <v>27.4999324615825</v>
       </c>
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="n">
@@ -10485,13 +10485,13 @@
         <v>1</v>
       </c>
       <c r="AC94" t="n">
-        <v>3.348948039188035</v>
+        <v>3.349901717502762</v>
       </c>
       <c r="AD94" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="AE94" t="n">
-        <v>3.295836866004329</v>
+        <v>2.772588722239781</v>
       </c>
     </row>
     <row r="95">
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>47.47276565028113</v>
+        <v>48.94968790033269</v>
       </c>
       <c r="C95" t="n">
         <v>0.74</v>
@@ -10592,13 +10592,13 @@
         <v>3</v>
       </c>
       <c r="AC95" t="n">
-        <v>3.881002107240852</v>
+        <v>3.911016256833455</v>
       </c>
       <c r="AD95" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="AE95" t="n">
-        <v>4.30406509320417</v>
+        <v>3.637586159726386</v>
       </c>
     </row>
     <row r="96">
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>86.47276565028113</v>
+        <v>85.91539457283963</v>
       </c>
       <c r="C96" t="n">
         <v>0.84</v>
@@ -10699,13 +10699,13 @@
         <v>8</v>
       </c>
       <c r="AC96" t="n">
-        <v>4.471327495204251</v>
+        <v>4.464935169318588</v>
       </c>
       <c r="AD96" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="AE96" t="n">
-        <v>2.772588722239781</v>
+        <v>2.484906649788</v>
       </c>
     </row>
     <row r="97">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>33.47276565028113</v>
+        <v>33.13624798209644</v>
       </c>
       <c r="C97" t="n">
         <v>0.5600000000000001</v>
@@ -10806,13 +10806,13 @@
         <v>7</v>
       </c>
       <c r="AC97" t="n">
-        <v>3.5401696108548</v>
+        <v>3.530359810392252</v>
       </c>
       <c r="AD97" t="n">
-        <v>163</v>
+        <v>42</v>
       </c>
       <c r="AE97" t="n">
-        <v>5.099866427824199</v>
+        <v>3.761200115693562</v>
       </c>
     </row>
     <row r="98">
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>75.47276565028113</v>
+        <v>74.59587993285848</v>
       </c>
       <c r="C98" t="n">
         <v>0.72</v>
@@ -10913,13 +10913,13 @@
         <v>10</v>
       </c>
       <c r="AC98" t="n">
-        <v>4.33693467287633</v>
+        <v>4.325401783457791</v>
       </c>
       <c r="AD98" t="n">
-        <v>181</v>
+        <v>48</v>
       </c>
       <c r="AE98" t="n">
-        <v>5.204006687076795</v>
+        <v>3.891820298110626</v>
       </c>
     </row>
     <row r="99">
@@ -10929,7 +10929,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>16.5340374274238</v>
+        <v>17.68994269759877</v>
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
@@ -11018,13 +11018,13 @@
         <v>5</v>
       </c>
       <c r="AC99" t="n">
-        <v>2.864143987726897</v>
+        <v>2.927985555523701</v>
       </c>
       <c r="AD99" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="AE99" t="n">
-        <v>3.526360524616162</v>
+        <v>2.19722457733622</v>
       </c>
     </row>
     <row r="100">
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>104.195507246406</v>
+        <v>98.23527070411768</v>
       </c>
       <c r="C100" t="inlineStr"/>
       <c r="D100" t="n">
@@ -11123,13 +11123,13 @@
         <v>1</v>
       </c>
       <c r="AC100" t="n">
-        <v>4.655820592608436</v>
+        <v>4.597493502550187</v>
       </c>
       <c r="AD100" t="n">
-        <v>2828</v>
+        <v>1564</v>
       </c>
       <c r="AE100" t="n">
-        <v>7.947678571301568</v>
+        <v>7.355641102974253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>